<commit_message>
Anchors: give kat-4 (immune load) a rank-1 anchor and let a source anchor multiple categories
Promoted the cumulative-antigen-exposure study to the kat-4 rank-1 anchor, and extended anchoring so one source can be the anchor for more than one concern category (the general vaccine-safety review now anchors both general-safety and vaccine-ingredient questions).
</commit_message>
<xml_diff>
--- a/data/knowledge_base_references.xlsx
+++ b/data/knowledge_base_references.xlsx
@@ -1821,6 +1821,11 @@
       <c r="B49" t="n">
         <v>1</v>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>rank-1 (kat-1 + kat-3)</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>Vaccine Safety: Myths and Misinformation.</t>
@@ -2314,6 +2319,11 @@
       </c>
       <c r="B65" t="n">
         <v>4</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>rank-1</t>
+        </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Anchors: guarantee every category anchor and allow multiple anchors per category
Reworked anchor injection so each designated anchor source contributes its most relevant passage (previously a multi-chunk source could crowd the others out). Collapsed the two-tier rank system into a single anchor level, and added second/third anchors to several categories (fertility, natural-immunity, ethics, immune-load, distrust, effectiveness, decision-conflict) from the existing corpus.
</commit_message>
<xml_diff>
--- a/data/knowledge_base_references.xlsx
+++ b/data/knowledge_base_references.xlsx
@@ -2390,7 +2390,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>rank-2</t>
+          <t>rank-1</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>rank-2</t>
+          <t>rank-1</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2785,6 +2785,11 @@
       <c r="B80" t="n">
         <v>5</v>
       </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>rank-1</t>
+        </is>
+      </c>
       <c r="D80" t="inlineStr">
         <is>
           <t>The impact of COVID-19 vaccines on fertility-A systematic review and meta-analysis.</t>
@@ -2877,6 +2882,11 @@
       <c r="B83" t="n">
         <v>6</v>
       </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>rank-1</t>
+        </is>
+      </c>
       <c r="D83" t="inlineStr">
         <is>
           <t>Long-term immunogenicity after measles vaccine vs. wild infection: an Italian retrospective cohort study</t>
@@ -3344,7 +3354,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>rank-2</t>
+          <t>rank-1</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3463,6 +3473,11 @@
       <c r="B102" t="n">
         <v>8</v>
       </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>rank-1</t>
+        </is>
+      </c>
       <c r="D102" t="inlineStr">
         <is>
           <t>Moral reflections on vaccines prepared from cells derived from aborted human fetuses.</t>
@@ -3828,7 +3843,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>rank-2</t>
+          <t>rank-1</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4252,7 +4267,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>rank-2</t>
+          <t>rank-1</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">

</xml_diff>

<commit_message>
Data: drop journal and year columns from reference list (already in the full citation)
</commit_message>
<xml_diff>
--- a/data/knowledge_base_references.xlsx
+++ b/data/knowledge_base_references.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I130"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,25 +451,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>dergi</t>
+          <t>pubmed_url</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>yil</t>
+          <t>kunye</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>pubmed_url</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>kunye</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>parca</t>
         </is>
@@ -487,20 +477,17 @@
           <t>A systematic literature review to clarify the concept of vaccine hesitancy.</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/35995837/</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Bussink-Voorend, D., Hautvast, J. L. A., Vandeberg, L., Visser, O., &amp; Hulscher, M. E. J. L. (2022). A systematic literature review to clarify the concept of vaccine hesitancy. Nature human behaviour, 6(12), 1634–1648. https://doi.org/10.1038/s41562-022-01431-6</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="G2" t="n">
         <v>125</v>
       </c>
     </row>
@@ -516,20 +503,17 @@
           <t>A systematic review on the psychological factors behind vaccine hesitancy in the COVID-19 era.</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12644076/</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Panico, F., De Biase, R., Catalano, L., Zappullo, I., D'Olimpio, F., Trojano, L., &amp; Sagliano, L. (2025). A systematic review on the psychological factors behind vaccine hesitancy in the COVID-19 era. Frontiers in public health, 13, 1711428. https://doi.org/10.3389/fpubh.2025.1711428</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="G3" t="n">
         <v>58</v>
       </c>
     </row>
@@ -545,20 +529,17 @@
           <t>Addressing Parental Vaccine Hesitancy towards Childhood Vaccines in the United States: A Systematic Literature Review of Communication Interventions and Strategies.</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC7712553/</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Olson, O., Berry, C., &amp; Kumar, N. (2020). Addressing Parental Vaccine Hesitancy towards Childhood Vaccines in the United States: A Systematic Literature Review of Communication Interventions and Strategies. Vaccines, 8(4), 590. https://doi.org/10.3390/vaccines8040590</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="G4" t="n">
         <v>97</v>
       </c>
     </row>
@@ -574,20 +555,17 @@
           <t>Addressing vaccine hesitancy: A systematic review comparing the efficacy of motivational versus educational interventions on vaccination uptake.</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC11942781/</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Labbé, S., Bacon, S. L., Wu, N., Ribeiro, P. A. B., Boucher, V. G., Stojanovic, J., Voisard, B., Deslauriers, F., Tremblay, N., Hébert-Auger, L., &amp; Lavoie, K. L. (2025). Addressing vaccine hesitancy: A systematic review comparing the efficacy of motivational versus educational interventions on vaccination uptake. Translational behavioral medicine, 15(1), ibae069. https://doi.org/10.1093/tbm/ibae069</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="G5" t="n">
         <v>57</v>
       </c>
     </row>
@@ -603,20 +581,17 @@
           <t>Advisory Committee on Immunization Practices Recommended Immunization Schedule for Children and Adolescents Aged 18 Years or Younger — United States, 2022</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>https://www.cdc.gov/mmwr/volumes/71/wr/pdfs/mm7107a2-H.pdf</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Advisory Committee onImmunization Practices Recommended Immuniza-tion Schedule for Children and Adolescents Aged 18Years or Younger – United States, 2022</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="G6" t="n">
         <v>17</v>
       </c>
     </row>
@@ -632,15 +607,12 @@
           <t>Ulusal Çocukluk Dönemi Aşılama Takvimi</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>T.C. Saglik Bakanligi, Halk Sagligi Genel Mudurlugu. (2025). Ulusal Cocukluk Donemi Asilama Takvimi. Ankara: T.C. Saglik Bakanligi. https://asi.saglik.gov.tr/</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="G7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -656,20 +628,17 @@
           <t>Barriers of Influenza Vaccination Intention and Behavior - A Systematic Review of Influenza Vaccine Hesitancy, 2005 - 2016.</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>2017</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/28125629/</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Schmid, P., Rauber, D., Betsch, C., Lidolt, G., &amp; Denker, M. L. (2017). Barriers of Influenza Vaccination Intention and Behavior - A Systematic Review of Influenza Vaccine Hesitancy, 2005 - 2016. PloS one, 12(1), e0170550. https://doi.org/10.1371/journal.pone.0170550</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="G8" t="n">
         <v>184</v>
       </c>
     </row>
@@ -685,17 +654,17 @@
           <t>Behavioural and Social Drivers of Vaccination: Tools and Practical Guidance for Achieving High Uptake</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://iris.who.int/server/api/core/bitstreams/c9f4a77a-001e-477d-a9d1-b05832820b64/content</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Behavioural and social drivers of vaccinationTools and practical guidance for achieving high uptake</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="G9" t="n">
         <v>204</v>
       </c>
     </row>
@@ -711,17 +680,17 @@
           <t>Catalogue of interventions addressing vaccine hesitancy</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>https://www.ecdc.europa.eu/sites/default/files/documents/Catalogue-interventions-vaccine-hesitancy.pdf</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Catalogue of interventions addressing vaccine hesitancy</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="G10" t="n">
         <v>159</v>
       </c>
     </row>
@@ -737,20 +706,17 @@
           <t>Communication interventions to reduce parental vaccine hesitancy: A systematic review.</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/40544799/</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Jwa, S., Imanishi, Y., Ascher, M. T., &amp; Dudley, M. Z. (2025). Communication interventions to reduce parental vaccine hesitancy: A systematic review. Vaccine, 61, 127401. https://doi.org/10.1016/j.vaccine.2025.127401</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="G11" t="n">
         <v>70</v>
       </c>
     </row>
@@ -766,20 +732,17 @@
           <t>Diagnosing the determinants of vaccine hesitancy in specific subgroups: The Guide to Tailoring Immunization Programmes (TIP).</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25896376/</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Butler, R., MacDonald, N. E., &amp; SAGE Working Group on Vaccine Hesitancy (2015). Diagnosing the determinants of vaccine hesitancy in specific subgroups: The Guide to Tailoring Immunization Programmes (TIP). Vaccine, 33(34), 4176–4179. https://doi.org/10.1016/j.vaccine.2015.04.038</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="G12" t="n">
         <v>30</v>
       </c>
     </row>
@@ -795,20 +758,17 @@
           <t>Drivers of and barriers to routine adult vaccination: A systematic literature review.</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/36197070/</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Eiden, A. L., Barratt, J., &amp; Nyaku, M. K. (2022). Drivers of and barriers to routine adult vaccination: A systematic literature review. Human vaccines &amp; immunotherapeutics, 18(6), 2127290. https://doi.org/10.1080/21645515.2022.2127290</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="G13" t="n">
         <v>81</v>
       </c>
     </row>
@@ -824,20 +784,17 @@
           <t>Effective Approaches to Combat Vaccine Hesitancy.</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/35213864/</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Tuckerman, J., Kaufman, J., &amp; Danchin, M. (2022). Effective Approaches to Combat Vaccine Hesitancy. The Pediatric infectious disease journal, 41(5), e243–e245. https://doi.org/10.1097/INF.0000000000003499</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="G14" t="n">
         <v>20</v>
       </c>
     </row>
@@ -853,20 +810,17 @@
           <t>Evidence-Based Strategies for Clinical Organizations to Address COVID-19 Vaccine Hesitancy.</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/33673921/</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Finney Rutten, L. J., Zhu, X., Leppin, A. L., Ridgeway, J. L., Swift, M. D., Griffin, J. M., St Sauver, J. L., Virk, A., &amp; Jacobson, R. M. (2021). Evidence-Based Strategies for Clinical Organizations to Address COVID-19 Vaccine Hesitancy. Mayo Clinic proceedings, 96(3), 699–707. https://doi.org/10.1016/j.mayocp.2020.12.024</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="G15" t="n">
         <v>35</v>
       </c>
     </row>
@@ -882,20 +836,17 @@
           <t>Factors associated with parents' hesitancy to vaccinate their children against COVID-19: The moderator role of parental anxiety.</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12618725/</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Richard, J., Dubé, A., Jbilou, J., &amp; Lachance-Grzela, M. (2025). Factors associated with parents' hesitancy to vaccinate their children against COVID-19: The moderator role of parental anxiety. Journal of health psychology, 30(13), 3998–4012. https://doi.org/10.1177/13591053251323502</t>
         </is>
       </c>
-      <c r="I16" t="n">
+      <c r="G16" t="n">
         <v>55</v>
       </c>
     </row>
@@ -911,20 +862,12 @@
           <t>General Best Practice Guidelines for Immunization (ACIP)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>CDC</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Centers for Disease Control and Prevention (ACIP). General Best Practice Guidelines for Immunization. https://www.cdc.gov/vaccines/hcp/acip-recs/general-recs/downloads/general-recs.pdf</t>
         </is>
       </c>
-      <c r="I17" t="n">
+      <c r="G17" t="n">
         <v>384</v>
       </c>
     </row>
@@ -940,20 +883,17 @@
           <t>How to deal with vaccine hesitancy?.</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25896378/</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Eskola, J., Duclos, P., Schuster, M., MacDonald, N. E., &amp; SAGE Working Group on Vaccine Hesitancy (2015). How to deal with vaccine hesitancy?. Vaccine, 33(34), 4215–4217. https://doi.org/10.1016/j.vaccine.2015.04.043</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="G18" t="n">
         <v>22</v>
       </c>
     </row>
@@ -969,17 +909,17 @@
           <t>Let’s Talk About Hesitancy: Enhancing Confidence in Vaccination and Uptake</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>https://www.ecdc.europa.eu/sites/default/files/media/en/publications/Publications/lets-talk-about-hesitancy-vaccination-guide.pdf</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Let’s talk about hesitancyEnhancing confidence in vaccination and uptake</t>
         </is>
       </c>
-      <c r="I19" t="n">
+      <c r="G19" t="n">
         <v>43</v>
       </c>
     </row>
@@ -997,23 +937,15 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Cureus</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/40792311/</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Khair, M., &amp; Irfan, B. (2025). Mpox in the Middle East and North Africa: Containment, Prevention, and Future Measures. Cureus, 17(7), e87758. https://doi.org/10.7759/cureus.87758</t>
         </is>
       </c>
-      <c r="I20" t="n">
+      <c r="G20" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1029,20 +961,17 @@
           <t>Psychosocial dimensions of vaccine hesitancy: A systematic review.</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/38988066/</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Rizzo, M., Gattino, S., Trombetta, T., Calandri, E., &amp; De Piccoli, N. (2024). Psychosocial dimensions of vaccine hesitancy: A systematic review. Journal of community psychology, 52(7), 857–876. https://doi.org/10.1002/jcop.23133</t>
         </is>
       </c>
-      <c r="I21" t="n">
+      <c r="G21" t="n">
         <v>73</v>
       </c>
     </row>
@@ -1058,20 +987,12 @@
           <t>Recommended Child and Adolescent Immunization Schedule, 0-18 years (United States)</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>CDC</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Centers for Disease Control and Prevention. Recommended Child and Adolescent Immunization Schedule, 0-18 years, United States. https://www.cdc.gov/vaccines/hcp/imz-schedules/downloads/child/0-18yrs-child-combined-schedule.pdf</t>
         </is>
       </c>
-      <c r="I22" t="n">
+      <c r="G22" t="n">
         <v>85</v>
       </c>
     </row>
@@ -1087,20 +1008,17 @@
           <t>What Contributes to COVID-19 Vaccine Hesitancy? A Systematic Review of the Psychological Factors Associated with COVID-19 Vaccine Hesitancy</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>https://www.mdpi.com/2076-393X/10/11/1777?utm_source=chatgpt.com</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Romate J, Rajkumar E, Gopi A, Abraham J, Rages J, Lakshmi R, Jesline J, Bhogle S. What Contributes to COVID-19 Vaccine Hesitancy? A Systematic Review of the Psychological Factors Associated with COVID-19 Vaccine Hesitancy. Vaccines. 2022; 10(11):1777. https://doi.org/10.3390/vaccines10111777</t>
         </is>
       </c>
-      <c r="I23" t="n">
+      <c r="G23" t="n">
         <v>80</v>
       </c>
     </row>
@@ -1116,17 +1034,17 @@
           <t>Strengthening Confidence in Vaccines, Demand for Immunization and Addressing Vaccine Hesitancy: Considerations for Frontline Health Workers</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://www.unicef.org/eca/media/35331/file/Guide%20for%20health%20workers%20on%20strengthening%20confidence%20in%20vaccines.pdf.pdf</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>STRENGTHENING CONFIDENCE IN VACCINES, DEMAND FOR IMMUNIZATION AND ADDRESSING VACCINE HESITANCYCONSIDERATIONS FOR FRONTLINE HEALTH WORKERS</t>
         </is>
       </c>
-      <c r="I24" t="n">
+      <c r="G24" t="n">
         <v>90</v>
       </c>
     </row>
@@ -1142,20 +1060,12 @@
           <t>Sosyal Pediatri Derneği — Rutin Dışı Aşı Önerileri</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Sosyal Pediatri Derneği</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Sosyal Pediatri Derneği. Rutin Dışı Aşı Önerileri. https://www.sosyalpediatri.org.tr/assets/files/asi-uygulamalari/au1.pdf</t>
         </is>
       </c>
-      <c r="I25" t="n">
+      <c r="G25" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1171,17 +1081,17 @@
           <t>Summary WHO SAGE conclusions and recommendations on Vaccine Hesitancy</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>https://www.who.int/docs/default-source/immunization/demand/summary-of-sage-vaccinehesitancy-en.pdf</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Summary WHO SAGE conclusions and recommendations on Vaccine Hesitancy</t>
         </is>
       </c>
-      <c r="I26" t="n">
+      <c r="G26" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1197,20 +1107,12 @@
           <t>T.C. Sağlık Bakanlığı — Çocukluk Dönemi Rutin Aşı Takvimi (2025)</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>T.C. Sağlık Bakanlığı</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>T.C. Sağlık Bakanlığı. Çocukluk Dönemi Rutin Aşı Takvimi, 2025. https://asi.saglik.gov.tr/depo/2025/asi_takvimi/asi_takvimi_2025.pdf</t>
         </is>
       </c>
-      <c r="I27" t="n">
+      <c r="G27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1226,15 +1128,12 @@
           <t>Tailoring Immunization Programmes (TIP)</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>2019</v>
-      </c>
-      <c r="H28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>World Health Organization Regional Office for Europe. (2019). Tailoring Immunization Programmes (TIP). Copenhagen: WHO Regional Office for Europe. https://www.who.int/europe/publications/i/item/9789289054492</t>
         </is>
       </c>
-      <c r="I28" t="n">
+      <c r="G28" t="n">
         <v>194</v>
       </c>
     </row>
@@ -1250,20 +1149,17 @@
           <t>The 5As: A practical taxonomy for the determinants of vaccine uptake.</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>2016</v>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/26672676/</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Thomson, A., Robinson, K., &amp; Vallée-Tourangeau, G. (2016). The 5As: A practical taxonomy for the determinants of vaccine uptake. Vaccine, 34(8), 1018–1024. https://doi.org/10.1016/j.vaccine.2015.11.065</t>
         </is>
       </c>
-      <c r="I29" t="n">
+      <c r="G29" t="n">
         <v>47</v>
       </c>
     </row>
@@ -1279,17 +1175,17 @@
           <t>The Guide to Tailoring Immunization Programmes (TIP)</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>https://iris.who.int/server/api/core/bitstreams/9529a709-e3ae-4347-8343-36c9af585df2/content</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>The Guide to TailoringImmunization Programmes (TIP)</t>
         </is>
       </c>
-      <c r="I30" t="n">
+      <c r="G30" t="n">
         <v>168</v>
       </c>
     </row>
@@ -1305,20 +1201,17 @@
           <t>The WHO Tailoring Immunization Programmes (TIP) approach: Review of implementation to date.</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>2018</v>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/29287678/</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Dubé, E., Leask, J., Wolff, B., Hickler, B., Balaban, V., Hosein, E., &amp; Habersaat, K. (2018). The WHO Tailoring Immunization Programmes (TIP) approach: Review of implementation to date. Vaccine, 36(11), 1509–1515. https://doi.org/10.1016/j.vaccine.2017.12.012</t>
         </is>
       </c>
-      <c r="I31" t="n">
+      <c r="G31" t="n">
         <v>39</v>
       </c>
     </row>
@@ -1334,17 +1227,17 @@
           <t>Tools and methods for promoting vaccination acceptance and uptake: a social and behavioural science approach</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>https://www.ecdc.europa.eu/sites/default/files/documents/vaccination-acceptance-uptake-tools-social-behavioural-science.pdf</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Tools and methods for promoting vaccination acceptance and uptake: a social and behavioural science approach</t>
         </is>
       </c>
-      <c r="I32" t="n">
+      <c r="G32" t="n">
         <v>137</v>
       </c>
     </row>
@@ -1362,23 +1255,15 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Frontiers in Public Health</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/38264254/</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Montero, D. A., Vidal, R. M., Velasco, J., Carreno, L. J., Torres, J. P., Benachi O., M. A., ... O'Ryan, M. (2024). Two centuries of vaccination: historical and conceptual approach and future perspectives. Frontiers in Public Health, 11, 1326154. https://doi.org/10.3389/fpubh.2023.1326154</t>
         </is>
       </c>
-      <c r="I33" t="n">
+      <c r="G33" t="n">
         <v>179</v>
       </c>
     </row>
@@ -1394,20 +1279,17 @@
           <t>Understanding Vaccine Hesitancy: Insights and Improvement Strategies Drawn from a Multi-Study Review.</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12567618/</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Brumbaugh, K. Q., Gellert, F., &amp; Mokdad, A. H. (2025). Understanding Vaccine Hesitancy: Insights and Improvement Strategies Drawn from a Multi-Study Review. Vaccines, 13(10), 1003. https://doi.org/10.3390/vaccines13101003</t>
         </is>
       </c>
-      <c r="I34" t="n">
+      <c r="G34" t="n">
         <v>65</v>
       </c>
     </row>
@@ -1423,20 +1305,17 @@
           <t>Understanding vaccine hesitancy around vaccines and vaccination from a global perspective: a systematic review of published literature, 2007-2012.</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24598724/</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Larson, H. J., Jarrett, C., Eckersberger, E., Smith, D. M., &amp; Paterson, P. (2014). Understanding vaccine hesitancy around vaccines and vaccination from a global perspective: a systematic review of published literature, 2007-2012. Vaccine, 32(19), 2150–2159. https://doi.org/10.1016/j.vaccine.2014.01.081</t>
         </is>
       </c>
-      <c r="I35" t="n">
+      <c r="G35" t="n">
         <v>54</v>
       </c>
     </row>
@@ -1452,12 +1331,12 @@
           <t>Vaccine Misinformation Management Field Guide: Guidance for Addressing a Global Infodemic and Fostering Demand for Immunization</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>VACCINE MISINFORMATION MANAGEMENT FIELD GUIDEGuidance for addressing a global infodemic and fostering demand for immunization</t>
         </is>
       </c>
-      <c r="I36" t="n">
+      <c r="G36" t="n">
         <v>87</v>
       </c>
     </row>
@@ -1473,20 +1352,17 @@
           <t>Vaccine Hesitancy: Contemporary Issues and Historical Background.</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/36298459/</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Nuwarda, R. F., Ramzan, I., Weekes, L., &amp; Kayser, V. (2022). Vaccine Hesitancy: Contemporary Issues and Historical Background. Vaccines, 10(10), 1595. https://doi.org/10.3390/vaccines10101595</t>
         </is>
       </c>
-      <c r="I37" t="n">
+      <c r="G37" t="n">
         <v>98</v>
       </c>
     </row>
@@ -1502,20 +1378,17 @@
           <t>Vaccine Hesitancy: Obstacles and Challenges.</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/36245801/</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Galagali, P. M., Kinikar, A. A., &amp; Kumar, V. S. (2022). Vaccine Hesitancy: Obstacles and Challenges. Current pediatrics reports, 10(4), 241–248. https://doi.org/10.1007/s40124-022-00278-9</t>
         </is>
       </c>
-      <c r="I38" t="n">
+      <c r="G38" t="n">
         <v>38</v>
       </c>
     </row>
@@ -1531,20 +1404,17 @@
           <t>Vaccine Literacy and Vaccination: A Systematic Review.</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/36866001/</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Zhang, E., Dai, Z., Wang, S., Wang, X., Zhang, X., &amp; Fang, Q. (2023). Vaccine Literacy and Vaccination: A Systematic Review. International journal of public health, 68, 1605606. https://doi.org/10.3389/ijph.2023.1605606</t>
         </is>
       </c>
-      <c r="I39" t="n">
+      <c r="G39" t="n">
         <v>39</v>
       </c>
     </row>
@@ -1562,23 +1432,15 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Vaccine</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25896383/</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>MacDonald, N. E. (2015). Vaccine hesitancy: Definition, scope and determinants. Vaccine, 33(34), 4161-4164. https://doi.org/10.1016/j.vaccine.2015.04.036</t>
         </is>
       </c>
-      <c r="I40" t="n">
+      <c r="G40" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1594,20 +1456,17 @@
           <t>Vaccine hesitancy: an overview.</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>2013</v>
-      </c>
-      <c r="G41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23584253/</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Dubé, E., Laberge, C., Guay, M., Bramadat, P., Roy, R., &amp; Bettinger, J. (2013). Vaccine hesitancy: an overview. Human vaccines &amp; immunotherapeutics, 9(8), 1763–1773. https://doi.org/10.4161/hv.24657</t>
         </is>
       </c>
-      <c r="I41" t="n">
+      <c r="G41" t="n">
         <v>79</v>
       </c>
     </row>
@@ -1623,20 +1482,17 @@
           <t>Worldwide Child Routine Vaccination Hesitancy Rate among Parents of Children Aged 0-6 Years: A Systematic Review and Meta-Analysis of Cross-Sectional Studies.</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/38250844/</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Abenova, M., Shaltynov, A., Jamedinova, U., &amp; Semenova, Y. (2023). Worldwide Child Routine Vaccination Hesitancy Rate among Parents of Children Aged 0-6 Years: A Systematic Review and Meta-Analysis of Cross-Sectional Studies. Vaccines, 12(1), 31. https://doi.org/10.3390/vaccines12010031</t>
         </is>
       </c>
-      <c r="I42" t="n">
+      <c r="G42" t="n">
         <v>58</v>
       </c>
     </row>
@@ -1657,20 +1513,17 @@
           <t>Adverse Effects of Vaccines: Evidence and Causality.</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>2011</v>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24624471/</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Stratton, K., Ford, A., Rusch, E., Clayton, E. W., Committee to Review Adverse Effects of Vaccines, &amp; Institute of Medicine (Eds.). (2011). Adverse Effects of Vaccines: Evidence and Causality. National Academies Press (US). https://doi.org/10.17226/13164</t>
         </is>
       </c>
-      <c r="I43" t="n">
+      <c r="G43" t="n">
         <v>2069</v>
       </c>
     </row>
@@ -1686,20 +1539,17 @@
           <t>Evidence Review of the Adverse Effects of COVID-19 Vaccination and Intramuscular Vaccine Administration.</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/39312602/</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>National Academies of Sciences, Engineering, and Medicine; Health and Medicine Division; Board on Population Health and Public Health Practice; Committee to Review Relevant Literature Regarding Adverse Events Associated with Vaccines, Rosenberg, D., Kumova, O. K., Stratton, K., &amp; Bass, A. R. (Eds.). (2024). Evidence Review of the Adverse Effects of COVID-19 Vaccination and Intramuscular Vaccine Administration. National Academies Press (US). https://doi.org/10.17226/27746</t>
         </is>
       </c>
-      <c r="I44" t="n">
+      <c r="G44" t="n">
         <v>828</v>
       </c>
     </row>
@@ -1715,15 +1565,12 @@
           <t>Immunogenicity and Safety Study of a Quadrivalent Meningococcal Conjugate Vaccine (MenACYW-TT) Administered Concomitantly With Routine Pediatric Vaccines in Healthy Infants and Toddlers (Study MET61; Clinical Study Protocol)</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H45" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>Sanofi Pasteur. (2023). Immunogenicity and Safety Study of a Quadrivalent Meningococcal Conjugate Vaccine (MenACYW-TT) Administered Concomitantly With Routine Pediatric Vaccines in Healthy Infants and Toddlers (Study MET61; Clinical Study Protocol). ClinicalTrials.gov Identifier: NCT03691610. https://clinicaltrials.gov/study/NCT03691610</t>
         </is>
       </c>
-      <c r="I45" t="n">
+      <c r="G45" t="n">
         <v>293</v>
       </c>
     </row>
@@ -1739,15 +1586,12 @@
           <t>Safety of Vaccines Used for Routine Immunization in the United States: An Update</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H46" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Gidengil, C., Goetz, M. B., Newberry, S., Maglione, M., Hall, O., Larkin, J., Motala, A., &amp; Hempel, S. (2021). Safety of Vaccines Used for Routine Immunization in the United States: An Update (Comparative Effectiveness Review No. 244). Rockville (MD): Agency for Healthcare Research and Quality (US). https://www.ncbi.nlm.nih.gov/books/NBK572041/</t>
         </is>
       </c>
-      <c r="I46" t="n">
+      <c r="G46" t="n">
         <v>3706</v>
       </c>
     </row>
@@ -1763,20 +1607,17 @@
           <t>Safety of vaccines used for routine immunization of U.S. children: a systematic review</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25086160/</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Maglione, M. A., Das, L., Raaen, L., Smith, A., Chari, R., Newberry, S., Shanman, R., Perry, T., Goetz, M. B., &amp; Gidengil, C. (2014). Safety of vaccines used for routine immunization of U.S. children: a systematic review. Pediatrics, 134(2), 325–337. https://doi.org/10.1542/peds.2014-1079</t>
         </is>
       </c>
-      <c r="I47" t="n">
+      <c r="G47" t="n">
         <v>45</v>
       </c>
     </row>
@@ -1794,23 +1635,15 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>The New England Journal of Medicine</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>1994</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/7969278/</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Peltola, H., Heinonen, O. P., Valle, M., Paunio, M., Virtanen, M., Karanko, V., &amp; Cantell, K. (1994). The elimination of indigenous measles, mumps, and rubella from Finland by a 12-year, two-dose vaccination program. The New England Journal of Medicine, 331(21), 1397-1402. https://doi.org/10.1056/NEJM199411243312101</t>
         </is>
       </c>
-      <c r="I48" t="n">
+      <c r="G48" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1831,20 +1664,17 @@
           <t>Vaccine Safety: Myths and Misinformation.</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC7090020/</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>Geoghegan, S., O'Callaghan, K. P., &amp; Offit, P. A. (2020). Vaccine Safety: Myths and Misinformation. Frontiers in microbiology, 11, 372. https://doi.org/10.3389/fmicb.2020.00372</t>
         </is>
       </c>
-      <c r="I49" t="n">
+      <c r="G49" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1860,20 +1690,17 @@
           <t>Vaccine safety: medical contraindications, myths, and risk communication.</t>
         </is>
       </c>
-      <c r="F50" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G50" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/26034253/</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Smith M. (2015). Vaccine safety: medical contraindications, myths, and risk communication. Pediatrics in review, 36(6), 227–238. https://doi.org/10.1542/pir.36-6-227</t>
         </is>
       </c>
-      <c r="I50" t="n">
+      <c r="G50" t="n">
         <v>48</v>
       </c>
     </row>
@@ -1889,20 +1716,17 @@
           <t>Association between thimerosal-containing vaccine and autism.</t>
         </is>
       </c>
-      <c r="F51" t="n">
-        <v>2003</v>
-      </c>
-      <c r="G51" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/14519711/</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>Hviid, A., Stellfeld, M., Wohlfahrt, J., &amp; Melbye, M. (2003). Association between thimerosal-containing vaccine and autism. JAMA, 290(13), 1763–1766. https://doi.org/10.1001/jama.290.13.1763</t>
         </is>
       </c>
-      <c r="I51" t="n">
+      <c r="G51" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1918,20 +1742,12 @@
           <t>Hviid et al. 2019 Vaccine-Autism Study: Much Ado About Nothing?</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Journal of Biotechnology and Biomedicine</t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H52" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Hammond, J. R., Varia, J., &amp; Hooker, B. (2025). Hviid et al. 2019 Vaccine-Autism Study: Much Ado About Nothing? Journal of Biotechnology and Biomedicine, 8, 118-140. https://doi.org/10.26502/jbb.2642-91280185</t>
         </is>
       </c>
-      <c r="I52" t="n">
+      <c r="G52" t="n">
         <v>119</v>
       </c>
     </row>
@@ -1947,20 +1763,17 @@
           <t>Immunization Safety Review: Vaccines and Autism.</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>2004</v>
-      </c>
-      <c r="G53" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/20669467/</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>Institute of Medicine (US) Immunization Safety Review Committee. (2004). Immunization Safety Review: Vaccines and Autism. National Academies Press (US). https://doi.org/10.17226/10997</t>
         </is>
       </c>
-      <c r="I53" t="n">
+      <c r="G53" t="n">
         <v>487</v>
       </c>
     </row>
@@ -1976,20 +1789,17 @@
           <t>Increasing exposure to antibody-stimulating proteins and polysaccharides in vaccines is not associated with risk of autism.</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>2013</v>
-      </c>
-      <c r="G54" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23545349/</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>DeStefano, F., Price, C. S., &amp; Weintraub, E. S. (2013). Increasing exposure to antibody-stimulating proteins and polysaccharides in vaccines is not associated with risk of autism. The Journal of pediatrics, 163(2), 561–567. https://doi.org/10.1016/j.jpeds.2013.02.001</t>
         </is>
       </c>
-      <c r="I54" t="n">
+      <c r="G54" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2010,20 +1820,17 @@
           <t>Measles, Mumps, Rubella Vaccination and Autism: A Nationwide Cohort Study.</t>
         </is>
       </c>
-      <c r="F55" t="n">
-        <v>2019</v>
-      </c>
-      <c r="G55" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/30831578/</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>Hviid, A., Hansen, J. V., Frisch, M., &amp; Melbye, M. (2019). Measles, Mumps, Rubella Vaccination and Autism: A Nationwide Cohort Study. Annals of internal medicine, 170(8), 513–520. https://doi.org/10.7326/M18-2101</t>
         </is>
       </c>
-      <c r="I55" t="n">
+      <c r="G55" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2044,20 +1851,17 @@
           <t>Vaccines are not associated with autism: an evidence-based meta-analysis of case-control and cohort studies.</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G56" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24814559/</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Taylor, L. E., Swerdfeger, A. L., &amp; Eslick, G. D. (2014). Vaccines are not associated with autism: an evidence-based meta-analysis of case-control and cohort studies. Vaccine, 32(29), 3623–3629. https://doi.org/10.1016/j.vaccine.2014.04.085</t>
         </is>
       </c>
-      <c r="I56" t="n">
+      <c r="G56" t="n">
         <v>40</v>
       </c>
     </row>
@@ -2073,20 +1877,17 @@
           <t>Vaccines for measles, mumps, rubella, and varicella in children.</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G57" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/34806766/</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>Di Pietrantonj, C., Rivetti, A., Marchione, P., Debalini, M. G., &amp; Demicheli, V. (2021). Vaccines for measles, mumps, rubella, and varicella in children. The Cochrane database of systematic reviews, 11(11), CD004407. https://doi.org/10.1002/14651858.CD004407.pub5</t>
         </is>
       </c>
-      <c r="I57" t="n">
+      <c r="G57" t="n">
         <v>1155</v>
       </c>
     </row>
@@ -2102,20 +1903,17 @@
           <t>Adverse events after immunisation with aluminium-containing DTP vaccines: systematic review of the evidence.</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>2004</v>
-      </c>
-      <c r="G58" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/14871632/</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>Jefferson, T., Rudin, M., &amp; Di Pietrantonj, C. (2004). Adverse events after immunisation with aluminium-containing DTP vaccines: systematic review of the evidence. The Lancet. Infectious diseases, 4(2), 84–90. https://doi.org/10.1016/S1473-3099(04)00927-2</t>
         </is>
       </c>
-      <c r="I58" t="n">
+      <c r="G58" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2133,23 +1931,15 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Biologicals</t>
-        </is>
-      </c>
-      <c r="F59" t="n">
-        <v>2009</v>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/19285882/</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Sheng-Fowler L, Lewis AM Jr, Peden K. Issues associated with residual cell-substrate DNA in viral vaccines. Biologicals. 2009;37(3):190-195.</t>
         </is>
       </c>
-      <c r="I59" t="n">
+      <c r="G59" t="n">
         <v>33</v>
       </c>
     </row>
@@ -2167,23 +1957,15 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Vaccine</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>2013</v>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23583892/</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>Mitkus RJ, Hess MA, Schwartz SL. Pharmacokinetic modeling as an approach to assessing the safety of residual formaldehyde in infant vaccines. Vaccine. 2013;31(27):2738-2743.</t>
         </is>
       </c>
-      <c r="I60" t="n">
+      <c r="G60" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2199,20 +1981,17 @@
           <t>Safety of thimerosal-containing vaccines: a two-phased study of computerized health maintenance organization databases.</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>2003</v>
-      </c>
-      <c r="G61" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/14595043/</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>Verstraeten, T., Davis, R. L., DeStefano, F., Lieu, T. A., Rhodes, P. H., Black, S. B., Shinefield, H., Chen, R. T., &amp; Vaccine Safety Datalink Team (2003). Safety of thimerosal-containing vaccines: a two-phased study of computerized health maintenance organization databases. Pediatrics, 112(5), 1039–1048.</t>
         </is>
       </c>
-      <c r="I61" t="n">
+      <c r="G61" t="n">
         <v>53</v>
       </c>
     </row>
@@ -2228,20 +2007,17 @@
           <t>Updated aluminum pharmacokinetics following infant exposures through diet and vaccination.</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>2011</v>
-      </c>
-      <c r="G62" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22001122/</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>Mitkus, R. J., King, D. B., Hess, M. A., Forshee, R. A., &amp; Walderhaug, M. O. (2011). Updated aluminum pharmacokinetics following infant exposures through diet and vaccination. Vaccine, 29(51), 9538–9543. https://doi.org/10.1016/j.vaccine.2011.09.124</t>
         </is>
       </c>
-      <c r="I62" t="n">
+      <c r="G62" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2259,23 +2035,15 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Nature Reviews Drug Discovery</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>2018</v>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/29326426/</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Pardi N, Hogan MJ, Porter FW, Weissman D. mRNA vaccines - a new era in vaccinology. Nature Reviews Drug Discovery. 2018;17(4):261-279.</t>
         </is>
       </c>
-      <c r="I63" t="n">
+      <c r="G63" t="n">
         <v>126</v>
       </c>
     </row>
@@ -2293,23 +2061,15 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Nature Reviews Drug Discovery</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/34433919/</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>Chaudhary N, Weissman D, Whitehead KA. mRNA vaccines for infectious diseases: principles, delivery and clinical translation. Nature Reviews Drug Discovery. 2021;20(11):817-838.</t>
         </is>
       </c>
-      <c r="I64" t="n">
+      <c r="G64" t="n">
         <v>137</v>
       </c>
     </row>
@@ -2330,20 +2090,17 @@
           <t>Association Between Estimated Cumulative Vaccine Antigen Exposure Through the First 23 Months of Life and Non-Vaccine-Targeted Infections From 24 Through 47 Months of Age.</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>2018</v>
-      </c>
-      <c r="G65" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/29509866/</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>Glanz, J. M., Newcomer, S. R., Daley, M. F., DeStefano, F., Groom, H. C., Jackson, M. L., Lewin, B. J., McCarthy, N. L., McClure, D. L., Narwaney, K. J., Nordin, J. D., &amp; Zerbo, O. (2018). Association Between Estimated Cumulative Vaccine Antigen Exposure Through the First 23 Months of Life and Non-Vaccine-Targeted Infections From 24 Through 47 Months of Age. JAMA, 319(9), 906–913. https://doi.org/10.1001/jama.2018.0708</t>
         </is>
       </c>
-      <c r="I65" t="n">
+      <c r="G65" t="n">
         <v>47</v>
       </c>
     </row>
@@ -2361,23 +2118,15 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Allergy</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/33569761/</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>Navaratna S, Estcourt MJ, Burgess J, et al. Childhood vaccination and allergy: A systematic review and meta-analysis. Allergy. 2021;76(7):2135-2152.</t>
         </is>
       </c>
-      <c r="I66" t="n">
+      <c r="G66" t="n">
         <v>76</v>
       </c>
     </row>
@@ -2398,20 +2147,17 @@
           <t>Childhood vaccination and nontargeted infectious disease hospitalization.</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>2005</v>
-      </c>
-      <c r="G67" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/16091572/</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>Hviid, A., Wohlfahrt, J., Stellfeld, M., &amp; Melbye, M. (2005). Childhood vaccination and nontargeted infectious disease hospitalization. JAMA, 294(6), 699–705. https://doi.org/10.1001/jama.294.6.699</t>
         </is>
       </c>
-      <c r="I67" t="n">
+      <c r="G67" t="n">
         <v>34</v>
       </c>
     </row>
@@ -2427,20 +2173,17 @@
           <t>On-time vaccine receipt in the first year does not adversely affect neuropsychological outcomes.</t>
         </is>
       </c>
-      <c r="F68" t="n">
-        <v>2010</v>
-      </c>
-      <c r="G68" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/20498176/</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>Smith, M. J., &amp; Woods, C. R. (2010). On-time vaccine receipt in the first year does not adversely affect neuropsychological outcomes. Pediatrics, 125(6), 1134–1141. https://doi.org/10.1542/peds.2009-2489</t>
         </is>
       </c>
-      <c r="I68" t="n">
+      <c r="G68" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2461,20 +2204,17 @@
           <t>The Childhood Immunization Schedule and Safety: Stakeholder Concerns, Scientific Evidence, and Future Studies.</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>2013</v>
-      </c>
-      <c r="G69" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24901198/</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>Committee on the Assessment of Studies of Health Outcomes Related to the Recommended Childhood Immunization Schedule, Board on Population Health and Public Health Practice, &amp; Institute of Medicine. (2013). The Childhood Immunization Schedule and Safety: Stakeholder Concerns, Scientific Evidence, and Future Studies. National Academies Press (US). https://doi.org/10.17226/13563</t>
         </is>
       </c>
-      <c r="I69" t="n">
+      <c r="G69" t="n">
         <v>572</v>
       </c>
     </row>
@@ -2490,20 +2230,17 @@
           <t>The problem with Dr Bob's alternative vaccine schedule.</t>
         </is>
       </c>
-      <c r="F70" t="n">
-        <v>2009</v>
-      </c>
-      <c r="G70" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/19117838/</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>Offit, P. A., &amp; Moser, C. A. (2009). The problem with Dr Bob's alternative vaccine schedule. Pediatrics, 123(1), e164–e169. https://doi.org/10.1542/peds.2008-2189</t>
         </is>
       </c>
-      <c r="I70" t="n">
+      <c r="G70" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2521,23 +2258,15 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Perspectives in Public Health</t>
-        </is>
-      </c>
-      <c r="F71" t="n">
-        <v>2016</v>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC4966430/</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>Bloomfield SF, Rook GA, Scott EA, Shanahan F, Stanwell-Smith R, Turner P. Time to abandon the hygiene hypothesis: new perspectives on allergic disease, the human microbiome, infectious disease prevention and the role of targeted hygiene. Perspectives in Public Health. 2016;136(4):213-224.</t>
         </is>
       </c>
-      <c r="I71" t="n">
+      <c r="G71" t="n">
         <v>72</v>
       </c>
     </row>
@@ -2553,20 +2282,17 @@
           <t>Association Between Human Papillomavirus Vaccination and Primary Ovarian Insufficiency in a Nationwide Cohort.</t>
         </is>
       </c>
-      <c r="F72" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G72" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/34436612/</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>Hviid, A., &amp; Myrup Thiesson, E. (2021). Association Between Human Papillomavirus Vaccination and Primary Ovarian Insufficiency in a Nationwide Cohort. JAMA network open, 4(8), e2120391. https://doi.org/10.1001/jamanetworkopen.2021.20391</t>
         </is>
       </c>
-      <c r="I72" t="n">
+      <c r="G72" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2582,20 +2308,17 @@
           <t>Effect of COVID-19 vaccination on the outcome of in vitro fertilization: A systematic review and meta-analysis.</t>
         </is>
       </c>
-      <c r="F73" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G73" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10106637/</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>Zhang, L., Sun, X., Wang, R., &amp; Ma, F. (2023). Effect of COVID-19 vaccination on the outcome of in vitro fertilization: A systematic review and meta-analysis. Frontiers in public health, 11, 1151999. https://doi.org/10.3389/fpubh.2023.1151999</t>
         </is>
       </c>
-      <c r="I73" t="n">
+      <c r="G73" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2611,20 +2334,17 @@
           <t>Effects of SARS-CoV-2 Vaccines on Sperm Quality: Systematic Review.</t>
         </is>
       </c>
-      <c r="F74" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G74" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10702876/</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>Li, G., Zhang, R., Song, B., Wang, C., Shen, Q., He, X., &amp; Cao, Y. (2023). Effects of SARS-CoV-2 Vaccines on Sperm Quality: Systematic Review. JMIR public health and surveillance, 9, e48511. https://doi.org/10.2196/48511</t>
         </is>
       </c>
-      <c r="I74" t="n">
+      <c r="G74" t="n">
         <v>66</v>
       </c>
     </row>
@@ -2640,20 +2360,17 @@
           <t>Primary Ovarian Insufficiency and Adolescent Vaccination.</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>2018</v>
-      </c>
-      <c r="G75" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/30131438/</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>Naleway, A. L., Mittendorf, K. F., Irving, S. A., Henninger, M. L., Crane, B., Smith, N., Daley, M. F., &amp; Gee, J. (2018). Primary Ovarian Insufficiency and Adolescent Vaccination. Pediatrics, 142(3), e20180943. https://doi.org/10.1542/peds.2018-0943</t>
         </is>
       </c>
-      <c r="I75" t="n">
+      <c r="G75" t="n">
         <v>35</v>
       </c>
     </row>
@@ -2669,20 +2386,17 @@
           <t>Risk of spontaneous abortion after mRNA COVID-19 vaccination received just prior to or during pregnancy: Complete data from CDC COVID-19 vaccine pregnancy registry.</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G76" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/41713234/</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>Madni, S. A., Olson, C. K., Zauche, L. H., Machefsky, A., Waters, A. V., Padathara-Mathew, R., Okereke, V., &amp; Sharma, A. J. (2026). Risk of spontaneous abortion after mRNA COVID-19 vaccination received just prior to or during pregnancy: Complete data from CDC COVID-19 vaccine pregnancy registry. Vaccine, 76, 128340. https://doi.org/10.1016/j.vaccine.2026.128340</t>
         </is>
       </c>
-      <c r="I76" t="n">
+      <c r="G76" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2698,20 +2412,17 @@
           <t>Safety of COVID-19 vaccines during pregnancy: A systematic review and meta-analysis.</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G77" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>http://pubmed.ncbi.nlm.nih.gov/37012114/</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>Ciapponi, A., Berrueta, M., P K Parker, E., Bardach, A., Mazzoni, A., Anderson, S. A., Argento, F. J., Ballivian, J., Bok, K., Comandé, D., Goucher, E., Kampmann, B., Munoz, F. M., Rodriguez Cairoli, F., Santa María, V., Stergachis, A. S., Voss, G., Xiong, X., Zamora, N., Zaraa, S., … Buekens, P. M. (2023). Safety of COVID-19 vaccines during pregnancy: A systematic review and meta-analysis. Vaccine, 41(25), 3688–3700. https://doi.org/10.1016/j.vaccine.2023.03.038</t>
         </is>
       </c>
-      <c r="I77" t="n">
+      <c r="G77" t="n">
         <v>90</v>
       </c>
     </row>
@@ -2732,20 +2443,17 @@
           <t>Systematic review and meta-analysis of the effectiveness and perinatal outcomes of COVID-19 vaccination in pregnancy.</t>
         </is>
       </c>
-      <c r="F78" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G78" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/35538060/</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>Prasad, S., Kalafat, E., Blakeway, H., Townsend, R., O'Brien, P., Morris, E., Draycott, T., Thangaratinam, S., Le Doare, K., Ladhani, S., von Dadelszen, P., Magee, L. A., Heath, P., &amp; Khalil, A. (2022). Systematic review and meta-analysis of the effectiveness and perinatal outcomes of COVID-19 vaccination in pregnancy. Nature communications, 13(1), 2414. https://doi.org/10.1038/s41467-022-30052-w</t>
         </is>
       </c>
-      <c r="I78" t="n">
+      <c r="G78" t="n">
         <v>48</v>
       </c>
     </row>
@@ -2761,20 +2469,17 @@
           <t>The effect of COVID-19 vaccines on sperm parameters: a systematic review and meta-analysis.</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G79" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/36510860/</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>Ma, Y. C., Cheng, C., Yuan, C., Xiang, L. Y., Wen, J., &amp; Jin, X. (2023). The effect of COVID-19 vaccines on sperm parameters: a systematic review and meta-analysis. Asian journal of andrology, 25(4), 468–473. https://doi.org/10.4103/aja2022100</t>
         </is>
       </c>
-      <c r="I79" t="n">
+      <c r="G79" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2795,20 +2500,17 @@
           <t>The impact of COVID-19 vaccines on fertility-A systematic review and meta-analysis.</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G80" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9464596/</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>Zaçe, D., La Gatta, E., Petrella, L., &amp; Di Pietro, M. L. (2022). The impact of COVID-19 vaccines on fertility-A systematic review and meta-analysis. Vaccine, 40(42), 6023–6034. https://doi.org/10.1016/j.vaccine.2022.09.019</t>
         </is>
       </c>
-      <c r="I80" t="n">
+      <c r="G80" t="n">
         <v>48</v>
       </c>
     </row>
@@ -2829,20 +2531,17 @@
           <t>Association Between Vaccine Refusal and Vaccine-Preventable Diseases in the United States: A Review of Measles and Pertussis.</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>2016</v>
-      </c>
-      <c r="G81" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC5007135/</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="F81" t="inlineStr">
         <is>
           <t>Phadke, V. K., Bednarczyk, R. A., Salmon, D. A., &amp; Omer, S. B. (2016). Association Between Vaccine Refusal and Vaccine-Preventable Diseases in the United States: A Review of Measles and Pertussis. JAMA, 315(11), 1149–1158. https://doi.org/10.1001/jama.2016.1353</t>
         </is>
       </c>
-      <c r="I81" t="n">
+      <c r="G81" t="n">
         <v>63</v>
       </c>
     </row>
@@ -2858,20 +2557,17 @@
           <t>Correlates of protection induced by vaccination.</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>2010</v>
-      </c>
-      <c r="G82" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/20463105/</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>Plotkin S. A. (2010). Correlates of protection induced by vaccination. Clinical and vaccine immunology : CVI, 17(7), 1055–1065. https://doi.org/10.1128/CVI.00131-10</t>
         </is>
       </c>
-      <c r="I82" t="n">
+      <c r="G82" t="n">
         <v>81</v>
       </c>
     </row>
@@ -2894,23 +2590,15 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Human Vaccines &amp; Immunotherapeutics</t>
-        </is>
-      </c>
-      <c r="F83" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC8189124/</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>Bianchi FP, Mascipinto S, Stefanizzi P, De Nitto S, Germinario C, Tafuri S. Long-term immunogenicity after measles vaccine vs. wild infection: an Italian retrospective cohort study. Human Vaccines &amp; Immunotherapeutics. 2021;17(7):2078-2084.</t>
         </is>
       </c>
-      <c r="I83" t="n">
+      <c r="G83" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2928,23 +2616,15 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Frontiers in Immunology</t>
-        </is>
-      </c>
-      <c r="F84" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25278941/</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>Niewiesk S. Maternal antibodies: clinical significance, mechanism of interference with immune responses, and possible vaccination strategies. Frontiers in Immunology. 2014;5:446.</t>
         </is>
       </c>
-      <c r="I84" t="n">
+      <c r="G84" t="n">
         <v>97</v>
       </c>
     </row>
@@ -2962,23 +2642,15 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Lancet</t>
-        </is>
-      </c>
-      <c r="F85" t="n">
-        <v>2017</v>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/28673424/</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="F85" t="inlineStr">
         <is>
           <t>Moss WJ. Measles. Lancet. 2017;390(10111):2490-2502.</t>
         </is>
       </c>
-      <c r="I85" t="n">
+      <c r="G85" t="n">
         <v>70</v>
       </c>
     </row>
@@ -2999,20 +2671,17 @@
           <t>Measles virus infection diminishes preexisting antibodies that offer protection from other pathogens.</t>
         </is>
       </c>
-      <c r="F86" t="n">
-        <v>2019</v>
-      </c>
-      <c r="G86" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/31672891/</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>Mina, M. J., Kula, T., Leng, Y., Li, M., de Vries, R. D., Knip, M., Siljander, H., Rewers, M., Choy, D. F., Wilson, M. S., Larman, H. B., Nelson, A. N., Griffin, D. E., de Swart, R. L., &amp; Elledge, S. J. (2019). Measles virus infection diminishes preexisting antibodies that offer protection from other pathogens. Science (New York, N.Y.), 366(6465), 599–606. https://doi.org/10.1126/science.aay6485</t>
         </is>
       </c>
-      <c r="I86" t="n">
+      <c r="G86" t="n">
         <v>49</v>
       </c>
     </row>
@@ -3028,20 +2697,17 @@
           <t>Parental refusal of pertussis vaccination is associated with an increased risk of pertussis infection in children.</t>
         </is>
       </c>
-      <c r="F87" t="n">
-        <v>2009</v>
-      </c>
-      <c r="G87" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/19482753/</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t>Glanz, J. M., McClure, D. L., Magid, D. J., Daley, M. F., France, E. K., Salmon, D. A., &amp; Hambidge, S. J. (2009). Parental refusal of pertussis vaccination is associated with an increased risk of pertussis infection in children. Pediatrics, 123(6), 1446–1451. https://doi.org/10.1542/peds.2008-2150</t>
         </is>
       </c>
-      <c r="I87" t="n">
+      <c r="G87" t="n">
         <v>35</v>
       </c>
     </row>
@@ -3057,20 +2723,17 @@
           <t>Parental refusal of varicella vaccination and the associated risk of varicella infection in children.</t>
         </is>
       </c>
-      <c r="F88" t="n">
-        <v>2010</v>
-      </c>
-      <c r="G88" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/20048244/</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>Glanz, J. M., McClure, D. L., Magid, D. J., Daley, M. F., France, E. K., &amp; Hambidge, S. J. (2010). Parental refusal of varicella vaccination and the associated risk of varicella infection in children. Archives of pediatrics &amp; adolescent medicine, 164(1), 66–70. https://doi.org/10.1001/archpediatrics.2009.244</t>
         </is>
       </c>
-      <c r="I88" t="n">
+      <c r="G88" t="n">
         <v>28</v>
       </c>
     </row>
@@ -3086,20 +2749,17 @@
           <t>Anti-vaccine activists, Web 2.0, and the postmodern paradigm--an overview of tactics and tropes used online by the anti-vaccination movement.</t>
         </is>
       </c>
-      <c r="F89" t="n">
-        <v>2012</v>
-      </c>
-      <c r="G89" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22172504/</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>Kata A. (2012). Anti-vaccine activists, Web 2.0, and the postmodern paradigm--an overview of tactics and tropes used online by the anti-vaccination movement. Vaccine, 30(25), 3778–3789. https://doi.org/10.1016/j.vaccine.2011.11.112</t>
         </is>
       </c>
-      <c r="I89" t="n">
+      <c r="G89" t="n">
         <v>104</v>
       </c>
     </row>
@@ -3115,20 +2775,17 @@
           <t>Beyond Tuskegee - Vaccine Distrust and Everyday Racism.</t>
         </is>
       </c>
-      <c r="F90" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G90" t="inlineStr">
+      <c r="E90" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/33471971/</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>Bajaj, S. S., &amp; Stanford, F. C. (2021). Beyond Tuskegee - Vaccine Distrust and Everyday Racism. The New England journal of medicine, 384(5), e12. https://doi.org/10.1056/NEJMpv2035827</t>
         </is>
       </c>
-      <c r="I90" t="n">
+      <c r="G90" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3144,20 +2801,17 @@
           <t>Compulsory vaccination and conscientious or philosophical exemptions: past, present, and future.</t>
         </is>
       </c>
-      <c r="F91" t="n">
-        <v>2006</v>
-      </c>
-      <c r="G91" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/16458770/</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>Salmon, D. A., Teret, S. P., MacIntyre, C. R., Salisbury, D., Burgess, M. A., &amp; Halsey, N. A. (2006). Compulsory vaccination and conscientious or philosophical exemptions: past, present, and future. Lancet (London, England), 367(9508), 436–442. https://doi.org/10.1016/S0140-6736(06)68144-0</t>
         </is>
       </c>
-      <c r="I91" t="n">
+      <c r="G91" t="n">
         <v>35</v>
       </c>
     </row>
@@ -3173,20 +2827,17 @@
           <t>Health consequences of religious and philosophical exemptions from immunization laws: individual and societal risk of measles.</t>
         </is>
       </c>
-      <c r="F92" t="n">
-        <v>1999</v>
-      </c>
-      <c r="G92" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/10404911/</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>Salmon, D. A., Haber, M., Gangarosa, E. J., Phillips, L., Smith, N. J., &amp; Chen, R. T. (1999). Health consequences of religious and philosophical exemptions from immunization laws: individual and societal risk of measles. JAMA, 282(1), 47–53. https://doi.org/10.1001/jama.282.1.47</t>
         </is>
       </c>
-      <c r="I92" t="n">
+      <c r="G92" t="n">
         <v>41</v>
       </c>
     </row>
@@ -3207,20 +2858,17 @@
           <t>Mapping global trends in vaccine confidence and investigating barriers to vaccine uptake: a large-scale retrospective temporal modelling study.</t>
         </is>
       </c>
-      <c r="F93" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G93" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/32919524/</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="F93" t="inlineStr">
         <is>
           <t>de Figueiredo, A., Simas, C., Karafillakis, E., Paterson, P., &amp; Larson, H. J. (2020). Mapping global trends in vaccine confidence and investigating barriers to vaccine uptake: a large-scale retrospective temporal modelling study. Lancet (London, England), 396(10255), 898–908. https://doi.org/10.1016/S0140-6736(20)31558-0</t>
         </is>
       </c>
-      <c r="I93" t="n">
+      <c r="G93" t="n">
         <v>51</v>
       </c>
     </row>
@@ -3236,20 +2884,17 @@
           <t>Measuring the impact of COVID-19 vaccine misinformation on vaccination intent in the UK and USA.</t>
         </is>
       </c>
-      <c r="F94" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G94" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/33547453/</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr">
+      <c r="F94" t="inlineStr">
         <is>
           <t>Loomba, S., de Figueiredo, A., Piatek, S. J., de Graaf, K., &amp; Larson, H. J. (2021). Measuring the impact of COVID-19 vaccine misinformation on vaccination intent in the UK and USA. Nature human behaviour, 5(3), 337–348. https://doi.org/10.1038/s41562-021-01056-1</t>
         </is>
       </c>
-      <c r="I94" t="n">
+      <c r="G94" t="n">
         <v>85</v>
       </c>
     </row>
@@ -3270,20 +2915,17 @@
           <t>The effects of anti-vaccine conspiracy theories on vaccination intentions.</t>
         </is>
       </c>
-      <c r="F95" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G95" t="inlineStr">
+      <c r="E95" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24586574/</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr">
+      <c r="F95" t="inlineStr">
         <is>
           <t>Jolley, D., &amp; Douglas, K. M. (2014). The effects of anti-vaccine conspiracy theories on vaccination intentions. PloS one, 9(2), e89177. https://doi.org/10.1371/journal.pone.0089177</t>
         </is>
       </c>
-      <c r="I95" t="n">
+      <c r="G95" t="n">
         <v>53</v>
       </c>
     </row>
@@ -3299,20 +2941,17 @@
           <t>The moral obligation to be vaccinated: utilitarianism, contractualism, and collective easy rescue.</t>
         </is>
       </c>
-      <c r="F96" t="n">
-        <v>2018</v>
-      </c>
-      <c r="G96" t="inlineStr">
+      <c r="E96" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/29429063/</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr">
+      <c r="F96" t="inlineStr">
         <is>
           <t>Giubilini, A., Douglas, T., &amp; Savulescu, J. (2018). The moral obligation to be vaccinated: utilitarianism, contractualism, and collective easy rescue. Medicine, health care, and philosophy, 21(4), 547–560. https://doi.org/10.1007/s11019-018-9829-y</t>
         </is>
       </c>
-      <c r="I96" t="n">
+      <c r="G96" t="n">
         <v>76</v>
       </c>
     </row>
@@ -3328,20 +2967,17 @@
           <t>Vaccine hesitancy: Definition, scope and determinants.</t>
         </is>
       </c>
-      <c r="F97" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G97" t="inlineStr">
+      <c r="E97" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25896383/</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr">
+      <c r="F97" t="inlineStr">
         <is>
           <t>MacDonald, N. E., &amp; SAGE Working Group on Vaccine Hesitancy (2015). Vaccine hesitancy: Definition, scope and determinants. Vaccine, 33(34), 4161–4164. https://doi.org/10.1016/j.vaccine.2015.04.036</t>
         </is>
       </c>
-      <c r="I97" t="n">
+      <c r="G97" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3362,20 +2998,17 @@
           <t>Vaccine refusal, mandatory immunization, and the risks of vaccine-preventable diseases.</t>
         </is>
       </c>
-      <c r="F98" t="n">
-        <v>2009</v>
-      </c>
-      <c r="G98" t="inlineStr">
+      <c r="E98" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/19420367/</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr">
+      <c r="F98" t="inlineStr">
         <is>
           <t>Omer, S. B., Salmon, D. A., Orenstein, W. A., deHart, M. P., &amp; Halsey, N. (2009). Vaccine refusal, mandatory immunization, and the risks of vaccine-preventable diseases. The New England journal of medicine, 360(19), 1981–1988. https://doi.org/10.1056/NEJMsa0806477</t>
         </is>
       </c>
-      <c r="I98" t="n">
+      <c r="G98" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3391,20 +3024,17 @@
           <t>Associations between religion, religiosity, and parental vaccine hesitancy.</t>
         </is>
       </c>
-      <c r="F99" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G99" t="inlineStr">
+      <c r="E99" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/34805968/</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr">
+      <c r="F99" t="inlineStr">
         <is>
           <t>Williams, J. T. B., Rice, J. D., &amp; O'Leary, S. T. (2021). Associations between religion, religiosity, and parental vaccine hesitancy. Vaccine: X, 9, 100121. https://doi.org/10.1016/j.jvacx.2021.100121</t>
         </is>
       </c>
-      <c r="I99" t="n">
+      <c r="G99" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3420,20 +3050,17 @@
           <t>Catholic Social Teaching and the Duty to Vaccinate.</t>
         </is>
       </c>
-      <c r="F100" t="n">
-        <v>2017</v>
-      </c>
-      <c r="G100" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/28328377/</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr">
+      <c r="F100" t="inlineStr">
         <is>
           <t>Carson, P. J., &amp; Flood, A. T. (2017). Catholic Social Teaching and the Duty to Vaccinate. The American journal of bioethics : AJOB, 17(4), 36–43. https://doi.org/10.1080/15265161.2017.1284914</t>
         </is>
       </c>
-      <c r="I100" t="n">
+      <c r="G100" t="n">
         <v>46</v>
       </c>
     </row>
@@ -3449,20 +3076,17 @@
           <t>Incidence of sexually transmitted infections after human papillomavirus vaccination among adolescent females.</t>
         </is>
       </c>
-      <c r="F101" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G101" t="inlineStr">
+      <c r="E101" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25664968/</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr">
+      <c r="F101" t="inlineStr">
         <is>
           <t>Jena, A. B., Goldman, D. P., &amp; Seabury, S. A. (2015). Incidence of sexually transmitted infections after human papillomavirus vaccination among adolescent females. JAMA internal medicine, 175(4), 617–623. https://doi.org/10.1001/jamainternmed.2014.7886</t>
         </is>
       </c>
-      <c r="I101" t="n">
+      <c r="G101" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3483,20 +3107,17 @@
           <t>Moral reflections on vaccines prepared from cells derived from aborted human fetuses.</t>
         </is>
       </c>
-      <c r="F102" t="n">
-        <v>2006</v>
-      </c>
-      <c r="G102" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/17091557/</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr">
+      <c r="F102" t="inlineStr">
         <is>
           <t>Pontifical Academy for Life (2006). Moral reflections on vaccines prepared from cells derived from aborted human fetuses. The national Catholic bioethics quarterly, 6(3), .</t>
         </is>
       </c>
-      <c r="I102" t="n">
+      <c r="G102" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3512,20 +3133,17 @@
           <t>Sexual activity-related outcomes after human papillomavirus vaccination of 11- to 12-year-olds.</t>
         </is>
       </c>
-      <c r="F103" t="n">
-        <v>2012</v>
-      </c>
-      <c r="G103" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23071201/</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr">
+      <c r="F103" t="inlineStr">
         <is>
           <t>Bednarczyk, R. A., Davis, R., Ault, K., Orenstein, W., &amp; Omer, S. B. (2012). Sexual activity-related outcomes after human papillomavirus vaccination of 11- to 12-year-olds. Pediatrics, 130(5), 798–805. https://doi.org/10.1542/peds.2012-1516</t>
         </is>
       </c>
-      <c r="I103" t="n">
+      <c r="G103" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3546,20 +3164,17 @@
           <t>Sharia (Islamic Law) Perspectives of COVID-19 Vaccines.</t>
         </is>
       </c>
-      <c r="F104" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G104" t="inlineStr">
+      <c r="E104" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/39574558/</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr">
+      <c r="F104" t="inlineStr">
         <is>
           <t>Mardian, Y., Shaw-Shaliba, K., Karyana, M., &amp; Lau, C. Y. (2021). Sharia (Islamic Law) Perspectives of COVID-19 Vaccines. Frontiers in tropical diseases, 2, 788188. https://doi.org/10.3389/fitd.2021.788188</t>
         </is>
       </c>
-      <c r="I104" t="n">
+      <c r="G104" t="n">
         <v>46</v>
       </c>
     </row>
@@ -3575,20 +3190,17 @@
           <t>THE ROLE OF ISTIHALAH (TRANSFORMATION) AND ISTIHLAK (CONSUMPTION) IN THE PERMISSIBILITY OF VACCINES DERIVED FROM FORBIDDEN ORIGINS: AN ISLAMIC LAW PERSPECTIVE.</t>
         </is>
       </c>
-      <c r="F105" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G105" t="inlineStr">
+      <c r="E105" t="inlineStr">
         <is>
           <t>https://dergipark.org.tr/en/pub/head/article/1338259</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr">
+      <c r="F105" t="inlineStr">
         <is>
           <t>Amin, A. M., &amp; Günay, H. M. (2023). THE ROLE OF ISTIHALAH (TRANSFORMATION) AND ISTIHLAK (CONSUMPTION) IN THE PERMISSIBILITY OF VACCINES DERIVED FROM FORBIDDEN ORIGINS: AN ISLAMIC LAW PERSPECTIVE. Helal Ve Etik Araştırmalar Dergisi, 5(2), 1-23. https://doi.org/10.51973/head.1338259</t>
         </is>
       </c>
-      <c r="I105" t="n">
+      <c r="G105" t="n">
         <v>83</v>
       </c>
     </row>
@@ -3604,20 +3216,17 @@
           <t>Vaccine hesitancy within the Muslim community: Islamic faith and public health perspectives.</t>
         </is>
       </c>
-      <c r="F106" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G106" t="inlineStr">
+      <c r="E106" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/36914409/</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr">
+      <c r="F106" t="inlineStr">
         <is>
           <t>Alsuwaidi, A. R., Hammad, H. A. A., Elbarazi, I., &amp; Sheek-Hussein, M. (2023). Vaccine hesitancy within the Muslim community: Islamic faith and public health perspectives. Human vaccines &amp; immunotherapeutics, 19(1), 2190716. https://doi.org/10.1080/21645515.2023.2190716</t>
         </is>
       </c>
-      <c r="I106" t="n">
+      <c r="G106" t="n">
         <v>44</v>
       </c>
     </row>
@@ -3638,20 +3247,17 @@
           <t>What the world's religions teach, applied to vaccines and immune globulins.</t>
         </is>
       </c>
-      <c r="F107" t="n">
-        <v>2013</v>
-      </c>
-      <c r="G107" t="inlineStr">
+      <c r="E107" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23499565/</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
+      <c r="F107" t="inlineStr">
         <is>
           <t>Grabenstein J. D. (2013). What the world's religions teach, applied to vaccines and immune globulins. Vaccine, 31(16), 2011–2023. https://doi.org/10.1016/j.vaccine.2013.02.026</t>
         </is>
       </c>
-      <c r="I107" t="n">
+      <c r="G107" t="n">
         <v>122</v>
       </c>
     </row>
@@ -3667,15 +3273,12 @@
           <t>Clarifying misconceptions in COVID-19 vaccine sentiment and stance analysis</t>
         </is>
       </c>
-      <c r="F108" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H108" t="inlineStr">
+      <c r="F108" t="inlineStr">
         <is>
           <t>Barberia, L. G., Lombard, B., Roman, N. T., &amp; Sousa, T. (2025). Clarifying misconceptions in COVID-19 vaccine sentiment and stance analysis. arXiv preprint arXiv:2503.18095. https://arxiv.org/abs/2503.18095</t>
         </is>
       </c>
-      <c r="I108" t="n">
+      <c r="G108" t="n">
         <v>47</v>
       </c>
     </row>
@@ -3696,20 +3299,17 @@
           <t>Social media and vaccine hesitancy.</t>
         </is>
       </c>
-      <c r="F109" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G109" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/33097547/</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>Wilson, S. L., &amp; Wiysonge, C. (2020). Social media and vaccine hesitancy. BMJ global health, 5(10), e004206. https://doi.org/10.1136/bmjgh-2020-004206</t>
         </is>
       </c>
-      <c r="I109" t="n">
+      <c r="G109" t="n">
         <v>36</v>
       </c>
     </row>
@@ -3725,20 +3325,17 @@
           <t>Social media and vaccine hesitancy: new updates for the era of COVID-19 and globalized infectious diseases.</t>
         </is>
       </c>
-      <c r="F110" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G110" t="inlineStr">
+      <c r="E110" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/32693678/</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr">
+      <c r="F110" t="inlineStr">
         <is>
           <t>Puri, N., Coomes, E. A., Haghbayan, H., &amp; Gunaratne, K. (2020). Social media and vaccine hesitancy: new updates for the era of COVID-19 and globalized infectious diseases. Human vaccines &amp; immunotherapeutics, 16(11), 2586–2593. https://doi.org/10.1080/21645515.2020.1780846</t>
         </is>
       </c>
-      <c r="I110" t="n">
+      <c r="G110" t="n">
         <v>46</v>
       </c>
     </row>
@@ -3759,20 +3356,17 @@
           <t>The impact of social networks on parents' vaccination decisions.</t>
         </is>
       </c>
-      <c r="F111" t="n">
-        <v>2013</v>
-      </c>
-      <c r="G111" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23589813/</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr">
+      <c r="F111" t="inlineStr">
         <is>
           <t>Brunson E. K. (2013). The impact of social networks on parents' vaccination decisions. Pediatrics, 131(5), e1397–e1404. https://doi.org/10.1542/peds.2012-2452</t>
         </is>
       </c>
-      <c r="I111" t="n">
+      <c r="G111" t="n">
         <v>38</v>
       </c>
     </row>
@@ -3788,20 +3382,17 @@
           <t>The influence of political ideology and trust on willingness to vaccinate.</t>
         </is>
       </c>
-      <c r="F112" t="n">
-        <v>2018</v>
-      </c>
-      <c r="G112" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/29370265/</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr">
+      <c r="F112" t="inlineStr">
         <is>
           <t>Baumgaertner, B., Carlisle, J. E., &amp; Justwan, F. (2018). The influence of political ideology and trust on willingness to vaccinate. PloS one, 13(1), e0191728. https://doi.org/10.1371/journal.pone.0191728</t>
         </is>
       </c>
-      <c r="I112" t="n">
+      <c r="G112" t="n">
         <v>45</v>
       </c>
     </row>
@@ -3817,20 +3408,17 @@
           <t>Vaccine hesitancy and behavior change theory-based social media interventions: a systematic review.</t>
         </is>
       </c>
-      <c r="F113" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G113" t="inlineStr">
+      <c r="E113" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/34850217/</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr">
+      <c r="F113" t="inlineStr">
         <is>
           <t>Li, L., Wood, C. E., &amp; Kostkova, P. (2022). Vaccine hesitancy and behavior change theory-based social media interventions: a systematic review. Translational behavioral medicine, 12(2), 243–272. https://doi.org/10.1093/tbm/ibab148</t>
         </is>
       </c>
-      <c r="I113" t="n">
+      <c r="G113" t="n">
         <v>105</v>
       </c>
     </row>
@@ -3853,23 +3441,15 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Clinical Infectious Diseases</t>
-        </is>
-      </c>
-      <c r="F114" t="n">
-        <v>2011</v>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/21427399/</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr">
+      <c r="F114" t="inlineStr">
         <is>
           <t>Fine, P., Eames, K., &amp; Heymann, D. L. (2011). "Herd immunity": a rough guide. Clinical infectious diseases, 52(7), 911-916. https://doi.org/10.1093/cid/cir007</t>
         </is>
       </c>
-      <c r="I114" t="n">
+      <c r="G114" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3892,23 +3472,15 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>The Journal of Infectious Diseases</t>
-        </is>
-      </c>
-      <c r="F115" t="n">
-        <v>2010</v>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/20402594/</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr">
+      <c r="F115" t="inlineStr">
         <is>
           <t>Weinberg, G. A., &amp; Szilagyi, P. G. (2010). Vaccine epidemiology: efficacy, effectiveness, and the translational research roadmap. The Journal of infectious diseases, 201(11), 1607-1610. https://doi.org/10.1086/652404</t>
         </is>
       </c>
-      <c r="I115" t="n">
+      <c r="G115" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3926,23 +3498,15 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Cochrane Database of Systematic Reviews</t>
-        </is>
-      </c>
-      <c r="F116" t="n">
-        <v>2012</v>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22336803/</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr">
+      <c r="F116" t="inlineStr">
         <is>
           <t>Demicheli, V., Rivetti, A., Debalini, M. G., &amp; Di Pietrantonj, C. (2012). Vaccines for measles, mumps and rubella in children. The Cochrane database of systematic reviews, 2012(2), CD004407. https://doi.org/10.1002/14651858.CD004407.pub3</t>
         </is>
       </c>
-      <c r="I116" t="n">
+      <c r="G116" t="n">
         <v>338</v>
       </c>
     </row>
@@ -3960,23 +3524,15 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>The New England Journal of Medicine</t>
-        </is>
-      </c>
-      <c r="F117" t="n">
-        <v>2012</v>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22970945/</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr">
+      <c r="F117" t="inlineStr">
         <is>
           <t>Klein, N. P., Bartlett, J., Rowhani-Rahbar, A., Fireman, B., &amp; Baxter, R. (2012). Waning protection after fifth dose of acellular pertussis vaccine in children. The New England journal of medicine, 367(11), 1012-1019. https://doi.org/10.1056/NEJMoa1200850</t>
         </is>
       </c>
-      <c r="I117" t="n">
+      <c r="G117" t="n">
         <v>33</v>
       </c>
     </row>
@@ -3997,20 +3553,17 @@
           <t>2013 IDSA clinical practice guideline for vaccination of the immunocompromised host.</t>
         </is>
       </c>
-      <c r="F118" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G118" t="inlineStr">
+      <c r="E118" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24421306/</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr">
+      <c r="F118" t="inlineStr">
         <is>
           <t>Rubin, L. G., Levin, M. J., Ljungman, P., Davies, E. G., Avery, R., Tomblyn, M., Bousvaros, A., Dhanireddy, S., Sung, L., Keyserling, H., Kang, I., &amp; Infectious Diseases Society of America (2014). 2013 IDSA clinical practice guideline for vaccination of the immunocompromised host. Clinical infectious diseases : an official publication of the Infectious Diseases Society of America, 58(3), 309–318. https://doi.org/10.1093/cid/cit816</t>
         </is>
       </c>
-      <c r="I118" t="n">
+      <c r="G118" t="n">
         <v>315</v>
       </c>
     </row>
@@ -4026,17 +3579,17 @@
           <t>ASCIA Guidelines - Vaccination of the Egg-Allergic Individual</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
+      <c r="E119" t="inlineStr">
         <is>
           <t>https://www.allergy.org.au/hp/papers/vaccination-of-the-egg-allergic-individual</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr">
+      <c r="F119" t="inlineStr">
         <is>
           <t>ASCIA Guidelines - Vaccination of the Egg-Allergic Individual</t>
         </is>
       </c>
-      <c r="I119" t="n">
+      <c r="G119" t="n">
         <v>28</v>
       </c>
     </row>
@@ -4054,23 +3607,15 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>JAMA</t>
-        </is>
-      </c>
-      <c r="F120" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/33683290/</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr">
+      <c r="F120" t="inlineStr">
         <is>
           <t>Blumenthal KG, Robinson LB, Camargo CA Jr, et al. Acute Allergic Reactions to mRNA COVID-19 Vaccines. JAMA. 2021;325(15):1562-1565.</t>
         </is>
       </c>
-      <c r="I120" t="n">
+      <c r="G120" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4091,20 +3636,17 @@
           <t>Adverse reactions to vaccines practice parameter 2012 update.</t>
         </is>
       </c>
-      <c r="F121" t="n">
-        <v>2012</v>
-      </c>
-      <c r="G121" t="inlineStr">
+      <c r="E121" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22608573/</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr">
+      <c r="F121" t="inlineStr">
         <is>
           <t>Kelso, J. M., Greenhawt, M. J., Li, J. T., Nicklas, R. A., Bernstein, D. I., Blessing-Moore, J., Cox, L., Khan, D., Lang, D. M., Oppenheimer, J., Portnoy, J. M., Randolph, C. R., Schuller, D. E., Spector, S. L., Tilles, S. A., &amp; Wallace, D. (2012). Adverse reactions to vaccines practice parameter 2012 update. The Journal of allergy and clinical immunology, 130(1), 25–43. https://doi.org/10.1016/j.jaci.2012.04.003</t>
         </is>
       </c>
-      <c r="I121" t="n">
+      <c r="G121" t="n">
         <v>105</v>
       </c>
     </row>
@@ -4120,20 +3662,17 @@
           <t>The adverse reactions to vaccines practice parameter 10 years on-what have we learned?.</t>
         </is>
       </c>
-      <c r="F122" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G122" t="inlineStr">
+      <c r="E122" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/35101646/</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr">
+      <c r="F122" t="inlineStr">
         <is>
           <t>Kelso J. M. (2022). The adverse reactions to vaccines practice parameter 10 years on-what have we learned?. Annals of allergy, asthma &amp; immunology : official publication of the American College of Allergy, Asthma, &amp; Immunology, 129(1), 35–39. https://doi.org/10.1016/j.anai.2022.01.026</t>
         </is>
       </c>
-      <c r="I122" t="n">
+      <c r="G122" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4149,20 +3688,17 @@
           <t>Clinician Communication to Address Vaccine Hesitancy.</t>
         </is>
       </c>
-      <c r="F123" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G123" t="inlineStr">
+      <c r="E123" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC11531800/</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr">
+      <c r="F123" t="inlineStr">
         <is>
           <t>Opel D. J. (2023). Clinician Communication to Address Vaccine Hesitancy. Pediatric clinics of North America, 70(2), 309–319. https://doi.org/10.1016/j.pcl.2022.11.008</t>
         </is>
       </c>
-      <c r="I123" t="n">
+      <c r="G123" t="n">
         <v>35</v>
       </c>
     </row>
@@ -4178,20 +3714,17 @@
           <t>Communicating with parents about vaccination: a framework for health professionals.</t>
         </is>
       </c>
-      <c r="F124" t="n">
-        <v>2012</v>
-      </c>
-      <c r="G124" t="inlineStr">
+      <c r="E124" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22998654/</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr">
+      <c r="F124" t="inlineStr">
         <is>
           <t>Leask, J., Kinnersley, P., Jackson, C., Cheater, F., Bedford, H., &amp; Rowles, G. (2012). Communicating with parents about vaccination: a framework for health professionals. BMC pediatrics, 12, 154. https://doi.org/10.1186/1471-2431-12-154</t>
         </is>
       </c>
-      <c r="I124" t="n">
+      <c r="G124" t="n">
         <v>56</v>
       </c>
     </row>
@@ -4207,20 +3740,17 @@
           <t>Effective messages in vaccine promotion: a randomized trial.</t>
         </is>
       </c>
-      <c r="F125" t="n">
-        <v>2014</v>
-      </c>
-      <c r="G125" t="inlineStr">
+      <c r="E125" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24590751/</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr">
+      <c r="F125" t="inlineStr">
         <is>
           <t>Nyhan, B., Reifler, J., Richey, S., &amp; Freed, G. L. (2014). Effective messages in vaccine promotion: a randomized trial. Pediatrics, 133(4), e835–e842. https://doi.org/10.1542/peds.2013-2365</t>
         </is>
       </c>
-      <c r="I125" t="n">
+      <c r="G125" t="n">
         <v>43</v>
       </c>
     </row>
@@ -4241,20 +3771,17 @@
           <t>Increasing Vaccination: Putting Psychological Science Into Action.</t>
         </is>
       </c>
-      <c r="F126" t="n">
-        <v>2017</v>
-      </c>
-      <c r="G126" t="inlineStr">
+      <c r="E126" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/29611455/</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr">
+      <c r="F126" t="inlineStr">
         <is>
           <t>Brewer, N. T., Chapman, G. B., Rothman, A. J., Leask, J., &amp; Kempe, A. (2017). Increasing Vaccination: Putting Psychological Science Into Action. Psychological science in the public interest : a journal of the American Psychological Society, 18(3), 149–207. https://doi.org/10.1177/1529100618760521</t>
         </is>
       </c>
-      <c r="I126" t="n">
+      <c r="G126" t="n">
         <v>310</v>
       </c>
     </row>
@@ -4275,20 +3802,17 @@
           <t>Motivational interviewing: A powerful tool to address vaccine hesitancy.</t>
         </is>
       </c>
-      <c r="F127" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G127" t="inlineStr">
+      <c r="E127" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC7145430/</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr">
+      <c r="F127" t="inlineStr">
         <is>
           <t>Gagneur A. (2020). Motivational interviewing: A powerful tool to address vaccine hesitancy. Canada communicable disease report = Releve des maladies transmissibles au Canada, 46(4), 93–97. https://doi.org/10.14745/ccdr.v46i04a06</t>
         </is>
       </c>
-      <c r="I127" t="n">
+      <c r="G127" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4304,20 +3828,17 @@
           <t>Promoting vaccination in maternity wards ─ motivational interview technique reduces hesitancy and enhances intention to vaccinate, results from a multicentre non-controlled pre- and post-intervention RCT-nested study, Quebec, March 2014 to February 2015.</t>
         </is>
       </c>
-      <c r="F128" t="n">
-        <v>2019</v>
-      </c>
-      <c r="G128" t="inlineStr">
+      <c r="E128" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC6737828/</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr">
+      <c r="F128" t="inlineStr">
         <is>
           <t>Gagneur, A., Battista, M. C., Boucher, F. D., Tapiero, B., Quach, C., De Wals, P., Lemaitre, T., Farrands, A., Boulianne, N., Sauvageau, C., Ouakki, M., Gosselin, V., Petit, G., Jacques, M. C., &amp; Dubé, È. (2019). Promoting vaccination in maternity wards ─ motivational interview technique reduces hesitancy and enhances intention to vaccinate, results from a multicentre non-controlled pre- and post-intervention RCT-nested study, Quebec, March 2014 to February 2015. Euro surveillance : bulletin Europeen sur les maladies transmissibles = European communicable disease bulletin, 24(36), 1800641. https://doi.org/10.2807/1560-7917.ES.2019.24.36.1800641</t>
         </is>
       </c>
-      <c r="I128" t="n">
+      <c r="G128" t="n">
         <v>55</v>
       </c>
     </row>
@@ -4333,20 +3854,17 @@
           <t>Strategies for Improving Vaccine Communication and Uptake.</t>
         </is>
       </c>
-      <c r="F129" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G129" t="inlineStr">
+      <c r="E129" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/38404211/</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr">
+      <c r="F129" t="inlineStr">
         <is>
           <t>O'Leary, S. T., Opel, D. J., Cataldi, J. R., Hackell, J. M., COMMITTEE ON INFECTIOUS DISEASES , COMMITTEE ON PRACTICE AND AMBULATORY MEDICINE , &amp; COMMITTEE ON BIOETHICS (2024). Strategies for Improving Vaccine Communication and Uptake. Pediatrics, 153(3), e2023065483. https://doi.org/10.1542/peds.2023-065483</t>
         </is>
       </c>
-      <c r="I129" t="n">
+      <c r="G129" t="n">
         <v>115</v>
       </c>
     </row>
@@ -4367,20 +3885,17 @@
           <t>The architecture of provider-parent vaccine discussions at health supervision visits.</t>
         </is>
       </c>
-      <c r="F130" t="n">
-        <v>2013</v>
-      </c>
-      <c r="G130" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24190677/</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr">
+      <c r="F130" t="inlineStr">
         <is>
           <t>Opel, D. J., Heritage, J., Taylor, J. A., Mangione-Smith, R., Salas, H. S., Devere, V., Zhou, C., &amp; Robinson, J. D. (2013). The architecture of provider-parent vaccine discussions at health supervision visits. Pediatrics, 132(6), 1037–1046. https://doi.org/10.1542/peds.2013-2037</t>
         </is>
       </c>
-      <c r="I130" t="n">
+      <c r="G130" t="n">
         <v>52</v>
       </c>
     </row>

</xml_diff>